<commit_message>
Daily oil & gas forecast 2026-09-26
</commit_message>
<xml_diff>
--- a/daily_forecasts/2026-09-26/oil_gas_price_forecast.xlsx
+++ b/daily_forecasts/2026-09-26/oil_gas_price_forecast.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Henry Hub ($/MMBtu)</t>
   </si>
   <si>
-    <t xml:space="preserve">Forecast made on prices up to 2026-09-25; 7 day = 2026-10-02, 15 day = 2026-10-12.</t>
+    <t xml:space="preserve">Forecast made on prices up to 2026-09-22; 7 day = 2026-09-29, 15 day = 2026-10-07.</t>
   </si>
   <si>
     <t xml:space="preserve">Prices in $/bbl except Henry Hub ($/MMBtu).</t>
@@ -643,7 +643,7 @@
       </c>
       <c r="I16" s="6" t="n">
         <f aca="false">Details!O2</f>
-        <v>0.953730645533371</v>
+        <v>0.953763672949448</v>
       </c>
       <c r="J16" s="5" t="n">
         <f aca="false">Details!G3</f>
@@ -651,7 +651,7 @@
       </c>
       <c r="K16" s="6" t="n">
         <f aca="false">Details!O3</f>
-        <v>0.931407571139562</v>
+        <v>0.931402196736894</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -664,7 +664,7 @@
       </c>
       <c r="I17" s="6" t="n">
         <f aca="false">Details!O4</f>
-        <v>0.954038854345771</v>
+        <v>0.954075921750053</v>
       </c>
       <c r="J17" s="5" t="n">
         <f aca="false">Details!G5</f>
@@ -672,7 +672,7 @@
       </c>
       <c r="K17" s="6" t="n">
         <f aca="false">Details!O5</f>
-        <v>0.931498322655786</v>
+        <v>0.931472286957467</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -685,7 +685,7 @@
       </c>
       <c r="I18" s="6" t="n">
         <f aca="false">Details!O6</f>
-        <v>0.890291007923315</v>
+        <v>0.890199965037576</v>
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">Details!G7</f>
@@ -693,7 +693,7 @@
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Details!O7</f>
-        <v>0.846987738187195</v>
+        <v>0.846827527911791</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -819,10 +819,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="E2" s="10" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="F2" s="11" t="n">
         <v>114.89</v>
@@ -835,35 +835,35 @@
         <v>0</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>103.160114889762</v>
+        <v>101.94825056334</v>
       </c>
       <c r="J2" s="11" t="n">
-        <v>127.104129195855</v>
+        <v>128.565264790535</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>95.0775464893845</v>
+        <v>93.1144400399458</v>
       </c>
       <c r="L2" s="11" t="n">
-        <v>134.836433701868</v>
+        <v>137.225317462959</v>
       </c>
       <c r="M2" s="13" t="n">
-        <v>0.530230326295585</v>
+        <v>0.531219980787704</v>
       </c>
       <c r="N2" s="14" t="n">
-        <v>0.0462693544666288</v>
+        <v>0.0462363270505519</v>
       </c>
       <c r="O2" s="15" t="n">
         <f aca="false">1-N2</f>
-        <v>0.953730645533371</v>
+        <v>0.953763672949448</v>
       </c>
       <c r="P2" s="13" t="n">
-        <v>0.693378119001919</v>
+        <v>0.6940441882805</v>
       </c>
       <c r="Q2" s="13" t="n">
-        <v>0.788955713504647</v>
+        <v>0.789272030651341</v>
       </c>
       <c r="R2" s="13" t="n">
-        <v>0.787644787644788</v>
+        <v>0.787234042553192</v>
       </c>
       <c r="S2" s="16" t="s">
         <v>31</v>
@@ -880,10 +880,10 @@
         <v>15</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="F3" s="11" t="n">
         <v>114.89</v>
@@ -896,35 +896,35 @@
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>97.2689137379789</v>
+        <v>95.509259484221</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>133.534447248019</v>
+        <v>135.762660795561</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>85.3484249090278</v>
+        <v>82.6121811734834</v>
       </c>
       <c r="L3" s="11" t="n">
-        <v>149.037593417766</v>
+        <v>153.35805542599</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>0.547641963426372</v>
+        <v>0.547687861271676</v>
       </c>
       <c r="N3" s="14" t="n">
-        <v>0.0685924288604382</v>
+        <v>0.0685978032631059</v>
       </c>
       <c r="O3" s="15" t="n">
         <f aca="false">1-N3</f>
-        <v>0.931407571139562</v>
+        <v>0.931402196736894</v>
       </c>
       <c r="P3" s="13" t="n">
-        <v>0.533686236766121</v>
+        <v>0.533718689788054</v>
       </c>
       <c r="Q3" s="13" t="n">
-        <v>0.794716565767749</v>
+        <v>0.79504132231405</v>
       </c>
       <c r="R3" s="13" t="n">
-        <v>0.779296875</v>
+        <v>0.778864970645792</v>
       </c>
       <c r="S3" s="16" t="s">
         <v>31</v>
@@ -941,10 +941,10 @@
         <v>7</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="F4" s="11" t="n">
         <v>96.41</v>
@@ -957,35 +957,35 @@
         <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>89.2919652387182</v>
+        <v>88.5392064656678</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>103.37407382841</v>
+        <v>104.172170454986</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>84.1205375159095</v>
+        <v>82.864404203947</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>107.32205803906</v>
+        <v>108.594045600806</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>0.534548944337812</v>
+        <v>0.535542747358309</v>
       </c>
       <c r="N4" s="14" t="n">
-        <v>0.0459611456542293</v>
+        <v>0.0459240782499474</v>
       </c>
       <c r="O4" s="15" t="n">
         <f aca="false">1-N4</f>
-        <v>0.954038854345771</v>
+        <v>0.954075921750053</v>
       </c>
       <c r="P4" s="13" t="n">
-        <v>0.699616122840691</v>
+        <v>0.700768491834774</v>
       </c>
       <c r="Q4" s="13" t="n">
-        <v>0.802624384909787</v>
+        <v>0.802408319649699</v>
       </c>
       <c r="R4" s="13" t="n">
-        <v>0.808880308880309</v>
+        <v>0.808510638297872</v>
       </c>
       <c r="S4" s="16" t="s">
         <v>31</v>
@@ -1002,10 +1002,10 @@
         <v>15</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>96.41</v>
@@ -1018,35 +1018,35 @@
         <v>0</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>85.8430630323128</v>
+        <v>84.7446636495265</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>106.536275403243</v>
+        <v>107.725208886862</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>78.2460999607669</v>
+        <v>76.4697250875054</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>114.015666990143</v>
+        <v>116.156894768211</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>0.554379210779596</v>
+        <v>0.554913294797688</v>
       </c>
       <c r="N5" s="14" t="n">
-        <v>0.0685016773442138</v>
+        <v>0.0685277130425333</v>
       </c>
       <c r="O5" s="15" t="n">
         <f aca="false">1-N5</f>
-        <v>0.931498322655786</v>
+        <v>0.931472286957467</v>
       </c>
       <c r="P5" s="13" t="n">
-        <v>0.534167468719923</v>
+        <v>0.534200385356455</v>
       </c>
       <c r="Q5" s="13" t="n">
-        <v>0.809025866813429</v>
+        <v>0.808264462809917</v>
       </c>
       <c r="R5" s="13" t="n">
-        <v>0.8125</v>
+        <v>0.812133072407045</v>
       </c>
       <c r="S5" s="16" t="s">
         <v>31</v>
@@ -1063,10 +1063,10 @@
         <v>7</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>2.9</v>
@@ -1079,35 +1079,35 @@
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>2.72572968164229</v>
+        <v>2.707254214317</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>3.09165992171546</v>
+        <v>3.11347801108038</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>2.60759652164454</v>
+        <v>2.57733467910111</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>3.25631417644535</v>
+        <v>3.29796668166094</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>0.497600767754319</v>
+        <v>0.498559077809798</v>
       </c>
       <c r="N6" s="14" t="n">
-        <v>0.109708992076685</v>
+        <v>0.109800034962424</v>
       </c>
       <c r="O6" s="15" t="n">
         <f aca="false">1-N6</f>
-        <v>0.890291007923315</v>
+        <v>0.890199965037576</v>
       </c>
       <c r="P6" s="13" t="n">
-        <v>0.421305182341651</v>
+        <v>0.420749279538905</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.819026790595954</v>
+        <v>0.818828680897646</v>
       </c>
       <c r="R6" s="13" t="n">
-        <v>0.83011583011583</v>
+        <v>0.829787234042553</v>
       </c>
       <c r="S6" s="16" t="s">
         <v>31</v>
@@ -1124,10 +1124,10 @@
         <v>15</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>2.9</v>
@@ -1140,35 +1140,35 @@
         <v>0</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>2.66699326800624</v>
+        <v>2.64261838305278</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>3.1692178362004</v>
+        <v>3.20101012672383</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2.51443811266479</v>
+        <v>2.4752416688381</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>3.4124115155948</v>
+        <v>3.48188203171248</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.487006737247353</v>
+        <v>0.486994219653179</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>0.153012261812805</v>
+        <v>0.153172472088209</v>
       </c>
       <c r="O7" s="15" t="n">
         <f aca="false">1-N7</f>
-        <v>0.846987738187195</v>
+        <v>0.846827527911791</v>
       </c>
       <c r="P7" s="13" t="n">
-        <v>0.296920115495669</v>
+        <v>0.295761078998073</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0.820583379196478</v>
+        <v>0.820936639118457</v>
       </c>
       <c r="R7" s="13" t="n">
-        <v>0.8125</v>
+        <v>0.812133072407045</v>
       </c>
       <c r="S7" s="16" t="s">
         <v>31</v>

</xml_diff>